<commit_message>
fix file BOM: add description for 221R
</commit_message>
<xml_diff>
--- a/03_BOM/Satellite_4U_Laser_Int_Ext_V110.xlsx
+++ b/03_BOM/Satellite_4U_Laser_Int_Ext_V110.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="196">
   <si>
     <t>Name</t>
   </si>
@@ -308,7 +308,7 @@
     <t>221R/1%</t>
   </si>
   <si>
-    <t>ERJ-3EKF2210V</t>
+    <t>RES SMD 221 OHM 1% 1/10W 0603</t>
   </si>
   <si>
     <t>R3</t>
@@ -611,7 +611,13 @@
     <t>CONV_TPS5430DDAR</t>
   </si>
   <si>
+    <t>Note</t>
+  </si>
+  <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Tô vàng: chưa có ở các board trước</t>
   </si>
 </sst>
 </file>
@@ -2049,7 +2055,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="19.6761904761905" customWidth="1"/>
@@ -3099,12 +3105,20 @@
       </c>
     </row>
     <row r="42" spans="1:8">
+      <c r="A42" t="s">
+        <v>193</v>
+      </c>
       <c r="C42" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D42">
         <f>SUM(D2:D40)</f>
         <v>172</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>